<commit_message>
Correct: Umbrella Task values written in full (no abbreviations); log lighting designer email sent + new RFI task
</commit_message>
<xml_diff>
--- a/260730_K5M_Task Tracker.xlsx
+++ b/260730_K5M_Task Tracker.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Task Tracker'!$A$10:$I$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Task Tracker'!$A$10:$I$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -532,12 +532,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="46" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
@@ -667,7 +667,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>MPFFE</t>
+          <t>Material Package FFE</t>
         </is>
       </c>
       <c r="D11" s="6" t="n">
@@ -708,7 +708,7 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>MPFFE</t>
+          <t>Material Package FFE</t>
         </is>
       </c>
       <c r="D12" s="6" t="n">
@@ -749,7 +749,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>FOSHD</t>
+          <t>Fitout SHD</t>
         </is>
       </c>
       <c r="D13" s="6" t="n">
@@ -790,7 +790,7 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>COMM-I</t>
+          <t>Communication Management - Internal</t>
         </is>
       </c>
       <c r="D14" s="6" t="n">
@@ -827,7 +827,7 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>SCOPE</t>
+          <t>Project Scope</t>
         </is>
       </c>
       <c r="D15" s="6" t="n">
@@ -872,7 +872,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>MPFFE</t>
+          <t>Material Package FFE</t>
         </is>
       </c>
       <c r="D16" s="6" t="n">
@@ -909,7 +909,7 @@
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>RFI-I</t>
+          <t>RFI - Internal</t>
         </is>
       </c>
       <c r="D17" s="6" t="n">
@@ -946,7 +946,7 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>FOSHD</t>
+          <t>Fitout SHD</t>
         </is>
       </c>
       <c r="D18" s="6" t="n">
@@ -991,7 +991,7 @@
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>FOSHD</t>
+          <t>Fitout SHD</t>
         </is>
       </c>
       <c r="D19" s="6" t="n">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>COC</t>
+          <t>COC Management</t>
         </is>
       </c>
       <c r="D20" s="6" t="n">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>WIPM</t>
+          <t>WDCO Internal Project Management</t>
         </is>
       </c>
       <c r="D21" s="6" t="n">
@@ -1106,7 +1106,7 @@
       </c>
       <c r="C22" s="6" t="inlineStr">
         <is>
-          <t>FSHD</t>
+          <t>FFE SHD</t>
         </is>
       </c>
       <c r="D22" s="6" t="n">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>MPFIT</t>
+          <t>Material Package Fitout</t>
         </is>
       </c>
       <c r="D23" s="6" t="n">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>WIPM</t>
+          <t>WDCO Internal Project Management</t>
         </is>
       </c>
       <c r="D24" s="6" t="n">
@@ -1225,7 +1225,7 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>MPFIT</t>
+          <t>Material Package Fitout</t>
         </is>
       </c>
       <c r="D25" s="6" t="n">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>COMM-C</t>
+          <t>Communication Management - Client</t>
         </is>
       </c>
       <c r="D26" s="6" t="n">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
@@ -1294,7 +1294,7 @@
       </c>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t>Per 29 Jul MoM, due today. Still need the designer's actual name/email for CONTACT_SHEET.md.</t>
+          <t>Introduction email sent 30 Jul. Still need the designer's actual name/email for CONTACT_SHEET.md.</t>
         </is>
       </c>
     </row>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>MPFFE</t>
+          <t>Material Package FFE</t>
         </is>
       </c>
       <c r="D27" s="6" t="n">
@@ -1339,13 +1339,58 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="inlineStr">
+        <is>
+          <t>Raise an RFI with the lighting designer</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>RFI - Client</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>Send an email</t>
+        </is>
+      </c>
+      <c r="F28" s="7" t="inlineStr">
+        <is>
+          <t>Shagun</t>
+        </is>
+      </c>
+      <c r="G28" s="6" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="H28" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="I28" s="7" t="inlineStr">
+        <is>
+          <t>Must close by 6 Aug. Specific RFI question/content not yet given — confirm what to ask her.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A10:I27"/>
+  <autoFilter ref="A10:I28"/>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
-  <conditionalFormatting sqref="G11:G27">
+  <conditionalFormatting sqref="G11:G28">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"To Do"</formula>
     </cfRule>
@@ -1357,19 +1402,19 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="5">
-    <dataValidation sqref="C11:C27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"SCOPE,SCHED,COMPL,FSHD,MPFFE,MPFIT,SPEC,RFI-C,RFI-I,RFI-PP,FOSHD,COC,COMM-I,COMM-PP,COMM-C,SITE,WIPM"</formula1>
+    <dataValidation sqref="C11:C28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Project Scope,Project Schedule,Compliance Collection,FFE SHD,Material Package FFE,Material Package Fitout,Specifications from client,RFI - Client,RFI - Internal,RFI - Production Partner,Fitout SHD,COC Management,Communication Management - Internal,Communication Management - Production Partner,Communication Management - Client,Site Survey Planning,WDCO Internal Project Management"</formula1>
     </dataValidation>
-    <dataValidation sqref="D11:D27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D11:D28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"1,2,3,4"</formula1>
     </dataValidation>
-    <dataValidation sqref="E11:E27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E11:E28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Documentation,Follow up call,Send an email,Follow up email,Arranging,Meeting online,Meeting physical"</formula1>
     </dataValidation>
-    <dataValidation sqref="F11:F27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F11:F28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Shagun,Claire,H&amp;T,Client,Ariel,Rahul,Other"</formula1>
     </dataValidation>
-    <dataValidation sqref="G11:G27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G11:G28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"To Do,In Progress,Done"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Fix row 14 data corruption from buggy append script; restore original task, correctly append new task at row 34; repair Status/Priority conditional-formatting ranges broken by earlier S.No. column insert
</commit_message>
<xml_diff>
--- a/260730_K5M_Task Tracker.xlsx
+++ b/260730_K5M_Task Tracker.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Task Tracker'!$A$10:$J$33</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Task Tracker'!$A$10:$K$34</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -379,7 +379,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -521,13 +521,25 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="17" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="15" fillId="6" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="15">
     <dxf>
       <font>
         <name val="Lato"/>
@@ -651,6 +663,72 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <font>
+        <color rgb="00FFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00A7A7A7"/>
+          <bgColor rgb="00A7A7A7"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="00292B2B"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFF07C"/>
+          <bgColor rgb="00FFF07C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="00FFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="0073BA9B"/>
+          <bgColor rgb="0073BA9B"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="00808080"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00D9D9D9"/>
+          <bgColor rgb="00D9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="00FFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E4572E"/>
+          <bgColor rgb="00E4572E"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="00FFFFFF"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="0026547C"/>
+          <bgColor rgb="0026547C"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -730,7 +808,7 @@
     <author>tc={75BFBEEB-3911-49E3-84BB-BBA5490465DD}</author>
   </authors>
   <commentList>
-    <comment ref="B15" authorId="0" shapeId="0">
+    <comment ref="C15" authorId="0" shapeId="0">
       <text>
         <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -963,10 +1041,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
     <col width="62" customWidth="1" min="2" max="2"/>
     <col width="31" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
@@ -979,1047 +1057,1152 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>K5M — TASK TRACKER</t>
-        </is>
-      </c>
-      <c r="J1" s="17" t="n"/>
+      <c r="K1" s="17" t="n"/>
     </row>
     <row r="2" ht="42" customHeight="1">
-      <c r="A2" s="16" t="inlineStr">
-        <is>
-          <t>v1 — 30 July 2026. Replaces the daily markdown task lists going forward — one continuous sheet, new rows appended as tasks come up (via #newtask) rather than a new file per day. '#GoodMorning' / '#ShowMeMyKanban' generates a Kanban view grouped by Status from this data.</t>
-        </is>
-      </c>
-      <c r="J2" s="16" t="n"/>
+      <c r="K2" s="16" t="n"/>
     </row>
     <row r="4" ht="24" customHeight="1">
-      <c r="A4" s="21" t="inlineStr">
-        <is>
-          <t>PRIORITY LEGEND</t>
-        </is>
-      </c>
+      <c r="A4" s="41" t="n"/>
       <c r="B4" s="41" t="n"/>
-      <c r="C4" s="3" t="n"/>
+      <c r="C4" s="41" t="n"/>
       <c r="D4" s="3" t="n"/>
       <c r="E4" s="3" t="n"/>
       <c r="F4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
+      <c r="G4" s="3" t="n"/>
       <c r="I4" s="3" t="n"/>
       <c r="J4" s="3" t="n"/>
+      <c r="K4" s="3" t="n"/>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="42" t="n">
+      <c r="B5" s="42" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Important and urgent</t>
         </is>
       </c>
-      <c r="C5" s="5" t="n"/>
       <c r="D5" s="5" t="n"/>
       <c r="E5" s="5" t="n"/>
-      <c r="F5" s="7" t="n"/>
-      <c r="H5" s="5" t="n"/>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="7" t="n"/>
       <c r="I5" s="5" t="n"/>
       <c r="J5" s="5" t="n"/>
+      <c r="K5" s="5" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="43" t="n">
+      <c r="B6" s="43" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>Urgent but not important</t>
         </is>
       </c>
-      <c r="C6" s="6" t="n"/>
       <c r="D6" s="6" t="n"/>
       <c r="E6" s="6" t="n"/>
-      <c r="F6" s="8" t="n"/>
-      <c r="H6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="8" t="n"/>
       <c r="I6" s="6" t="n"/>
       <c r="J6" s="6" t="n"/>
+      <c r="K6" s="6" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="44" t="n">
+      <c r="B7" s="44" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Important but not urgent</t>
         </is>
       </c>
-      <c r="C7" s="5" t="n"/>
       <c r="D7" s="5" t="n"/>
       <c r="E7" s="5" t="n"/>
-      <c r="F7" s="7" t="n"/>
-      <c r="H7" s="5" t="n"/>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="7" t="n"/>
       <c r="I7" s="5" t="n"/>
       <c r="J7" s="5" t="n"/>
+      <c r="K7" s="5" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="45" t="n">
+      <c r="B8" s="45" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>Neither — just needs a place to live</t>
         </is>
       </c>
-      <c r="C8" s="6" t="n"/>
       <c r="D8" s="6" t="n"/>
       <c r="E8" s="6" t="n"/>
-      <c r="F8" s="8" t="n"/>
-      <c r="H8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="8" t="n"/>
       <c r="I8" s="6" t="n"/>
       <c r="J8" s="6" t="n"/>
+      <c r="K8" s="6" t="n"/>
     </row>
     <row r="9" ht="8" customHeight="1"/>
     <row r="10" ht="26" customHeight="1" thickBot="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
+          <t>S.No.</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
           <t>Date Raised</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="C10" s="4" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>Umbrella Task</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="E10" s="4" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="F10" s="4" t="inlineStr">
         <is>
           <t>Type of Task</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>Dependent On 1</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>Dependent On 2</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="J10" s="4" t="inlineStr">
         <is>
           <t>Due/Target Date</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="K10" s="4" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="26" t="inlineStr">
+      <c r="A11" s="49" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="B11" s="37" t="inlineStr">
+      <c r="C11" s="37" t="inlineStr">
         <is>
           <t>Discuss with Claire — Material Package packaging (Claire vs Khamille)</t>
         </is>
       </c>
-      <c r="C11" s="34" t="inlineStr">
+      <c r="D11" s="34" t="inlineStr">
         <is>
           <t>Material Package FFE</t>
         </is>
       </c>
-      <c r="D11" s="39" t="n">
+      <c r="E11" s="39" t="n">
         <v>3</v>
       </c>
-      <c r="E11" s="19" t="inlineStr">
+      <c r="F11" s="19" t="inlineStr">
         <is>
           <t>Meeting physical</t>
         </is>
       </c>
-      <c r="F11" s="18" t="inlineStr">
+      <c r="G11" s="18" t="inlineStr">
         <is>
           <t>Claire</t>
         </is>
       </c>
-      <c r="G11" s="18" t="n"/>
-      <c r="H11" s="18" t="inlineStr">
+      <c r="H11" s="18" t="n"/>
+      <c r="I11" s="18" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I11" s="19" t="inlineStr"/>
-      <c r="J11" s="19" t="inlineStr">
+      <c r="J11" s="19" t="inlineStr"/>
+      <c r="K11" s="19" t="inlineStr">
         <is>
           <t>Resolved via 29 Jul MoM.</t>
         </is>
       </c>
-      <c r="K11" s="20" t="n"/>
+      <c r="L11" s="20" t="n"/>
     </row>
     <row r="12" ht="24" customHeight="1" thickBot="1">
-      <c r="A12" s="33" t="inlineStr">
+      <c r="A12" s="49" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" s="33" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="B12" s="38" t="inlineStr">
+      <c r="C12" s="38" t="inlineStr">
         <is>
           <t>Follow up with Khamille on sample presentation format &amp; timeline</t>
         </is>
       </c>
-      <c r="C12" s="35" t="inlineStr">
+      <c r="D12" s="35" t="inlineStr">
         <is>
           <t>Material Package FFE</t>
         </is>
       </c>
-      <c r="D12" s="10" t="n">
+      <c r="E12" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="8" t="inlineStr">
+      <c r="F12" s="8" t="inlineStr">
         <is>
           <t>Follow up call</t>
         </is>
       </c>
-      <c r="F12" s="23" t="inlineStr">
+      <c r="G12" s="23" t="inlineStr">
         <is>
           <t>Khamille</t>
         </is>
       </c>
-      <c r="G12" s="18" t="n"/>
-      <c r="H12" s="10" t="inlineStr">
+      <c r="H12" s="18" t="n"/>
+      <c r="I12" s="10" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="I12" s="10" t="inlineStr"/>
-      <c r="J12" s="8" t="inlineStr">
+      <c r="J12" s="10" t="inlineStr"/>
+      <c r="K12" s="8" t="inlineStr">
         <is>
           <t>Per 29 Jul MoM — explicitly flagged High priority, must not slip.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="26" t="inlineStr">
+      <c r="A13" s="49" t="n">
+        <v>3</v>
+      </c>
+      <c r="B13" s="26" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="B13" s="30" t="inlineStr">
+      <c r="C13" s="30" t="inlineStr">
         <is>
           <t>Discuss with Claire — fit-out substructure requirement approach</t>
         </is>
       </c>
-      <c r="C13" s="27" t="inlineStr">
+      <c r="D13" s="27" t="inlineStr">
         <is>
           <t>Fitout SHD</t>
         </is>
       </c>
-      <c r="D13" s="9" t="n">
+      <c r="E13" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>Meeting physical</t>
         </is>
       </c>
-      <c r="F13" s="9" t="n"/>
-      <c r="G13" s="18" t="n"/>
-      <c r="H13" s="9" t="inlineStr">
+      <c r="G13" s="9" t="n"/>
+      <c r="H13" s="18" t="n"/>
+      <c r="I13" s="9" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="I13" s="9" t="inlineStr"/>
-      <c r="J13" s="7" t="inlineStr">
+      <c r="J13" s="9" t="inlineStr"/>
+      <c r="K13" s="7" t="inlineStr">
         <is>
           <t>Not explicitly closed by the 29 Jul MoM — confirm still open.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="26" t="n"/>
-      <c r="B14" s="31" t="inlineStr">
+      <c r="A14" s="46" t="n">
+        <v>4</v>
+      </c>
+      <c r="B14" s="50" t="inlineStr"/>
+      <c r="C14" s="51" t="inlineStr">
         <is>
           <t xml:space="preserve">Send K5M "The Client" substrcture requirements for the fitout </t>
         </is>
       </c>
-      <c r="C14" s="28" t="inlineStr">
+      <c r="D14" s="51" t="inlineStr">
         <is>
           <t>RFI - Client</t>
         </is>
       </c>
-      <c r="D14" s="9" t="n">
+      <c r="E14" s="50" t="n">
         <v>1</v>
       </c>
-      <c r="E14" s="7" t="n"/>
-      <c r="F14" s="9" t="inlineStr">
+      <c r="F14" s="51" t="inlineStr"/>
+      <c r="G14" s="51" t="inlineStr">
         <is>
           <t>H&amp;T</t>
         </is>
       </c>
-      <c r="G14" s="18" t="n"/>
-      <c r="H14" s="9" t="inlineStr">
+      <c r="H14" s="47" t="inlineStr"/>
+      <c r="I14" s="50" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="I14" s="25" t="n">
+      <c r="J14" s="52" t="n">
         <v>46270</v>
       </c>
-      <c r="J14" s="7" t="n"/>
+      <c r="K14" s="51" t="inlineStr"/>
     </row>
     <row r="15" ht="24" customHeight="1" thickBot="1">
-      <c r="A15" s="26" t="n"/>
-      <c r="B15" s="32" t="inlineStr">
+      <c r="A15" s="49" t="n">
+        <v>5</v>
+      </c>
+      <c r="B15" s="26" t="n"/>
+      <c r="C15" s="32" t="inlineStr">
         <is>
           <t>Get Fitout Specification Drawings ready for supplier review / talk to Ariel about scaling and improving the fit-out drawing</t>
         </is>
       </c>
-      <c r="C15" s="28" t="inlineStr">
+      <c r="D15" s="28" t="inlineStr">
         <is>
           <t>Fitout SHD</t>
         </is>
       </c>
-      <c r="D15" s="9" t="n">
+      <c r="E15" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="F15" s="7" t="inlineStr">
         <is>
           <t>Follow up email</t>
         </is>
       </c>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="G15" s="9" t="inlineStr">
         <is>
           <t>Ariel</t>
         </is>
       </c>
-      <c r="G15" s="18" t="n"/>
-      <c r="H15" s="9" t="inlineStr">
+      <c r="H15" s="18" t="n"/>
+      <c r="I15" s="9" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n"/>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="9" t="n"/>
+      <c r="K15" s="24" t="inlineStr">
         <is>
           <t>Need to follow up with ariel to get deadline and quote  same as row no. 15</t>
         </is>
       </c>
     </row>
     <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="49" t="n">
+        <v>6</v>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="B16" s="29" t="inlineStr">
+      <c r="C16" s="29" t="inlineStr">
         <is>
           <t>Build project contact sheet (security log)</t>
         </is>
       </c>
-      <c r="C16" s="8" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>Communication Management - Internal</t>
         </is>
       </c>
-      <c r="D16" s="10" t="n">
+      <c r="E16" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E16" s="8" t="inlineStr">
+      <c r="F16" s="8" t="inlineStr">
         <is>
           <t>Documentation</t>
         </is>
       </c>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="18" t="n"/>
-      <c r="H16" s="10" t="inlineStr">
+      <c r="G16" s="10" t="n"/>
+      <c r="H16" s="18" t="n"/>
+      <c r="I16" s="10" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I16" s="10" t="inlineStr"/>
-      <c r="J16" s="8" t="inlineStr"/>
+      <c r="J16" s="10" t="inlineStr"/>
+      <c r="K16" s="8" t="inlineStr"/>
     </row>
     <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="9" t="inlineStr">
+      <c r="A17" s="49" t="n">
+        <v>7</v>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>Close the BOQ gap problem / Fit-out scope</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>Project Scope</t>
         </is>
       </c>
-      <c r="D17" s="9" t="n">
+      <c r="E17" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>Meeting physical</t>
         </is>
       </c>
-      <c r="F17" s="9" t="n"/>
-      <c r="G17" s="18" t="n"/>
-      <c r="H17" s="9" t="inlineStr">
+      <c r="G17" s="9" t="n"/>
+      <c r="H17" s="18" t="n"/>
+      <c r="I17" s="9" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="I17" s="9" t="inlineStr">
+      <c r="J17" s="9" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="J17" s="7" t="inlineStr">
+      <c r="K17" s="7" t="inlineStr">
         <is>
           <t>Stakeholder meeting scheduled Monday per 29 Jul MoM; no scope additions until then. Agenda topics confirmed 30 Jul: stone arch over wardrobe and fitted sofa, suspended glass light over the basin, fittings — hardware &amp; bathroom. See meetings/260803_K5M_Meeting_BOQ_Scope_Gap/pre-meeting/agenda.md.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="A18" s="49" t="n">
+        <v>8</v>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>Fix a meeting with H&amp;T — Material Package briefing</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="D18" s="8" t="inlineStr">
         <is>
           <t>Material Package FFE</t>
         </is>
       </c>
-      <c r="D18" s="10" t="n">
+      <c r="E18" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="E18" s="8" t="inlineStr">
+      <c r="F18" s="8" t="inlineStr">
         <is>
           <t>Meeting online</t>
         </is>
       </c>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="18" t="n"/>
-      <c r="H18" s="10" t="inlineStr">
+      <c r="G18" s="10" t="n"/>
+      <c r="H18" s="18" t="n"/>
+      <c r="I18" s="10" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I18" s="23" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">30th July </t>
         </is>
       </c>
-      <c r="J18" s="40" t="inlineStr">
+      <c r="K18" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">Meeting set at 10 am </t>
         </is>
       </c>
     </row>
     <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="23" t="inlineStr">
+      <c r="A19" s="49" t="n">
+        <v>9</v>
+      </c>
+      <c r="B19" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">29th july </t>
         </is>
       </c>
-      <c r="B19" s="40" t="inlineStr">
+      <c r="C19" s="40" t="inlineStr">
         <is>
           <t xml:space="preserve">Make an agenda for the HT material package review meeting. </t>
         </is>
       </c>
-      <c r="C19" s="8" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>Communication Management - Production Partner</t>
         </is>
       </c>
-      <c r="D19" s="10" t="n">
+      <c r="E19" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="E19" s="8" t="inlineStr">
+      <c r="F19" s="8" t="inlineStr">
         <is>
           <t>Documentation</t>
         </is>
       </c>
-      <c r="F19" s="10" t="n"/>
-      <c r="G19" s="18" t="n"/>
-      <c r="H19" s="10" t="inlineStr">
+      <c r="G19" s="10" t="n"/>
+      <c r="H19" s="18" t="n"/>
+      <c r="I19" s="10" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="I19" s="23" t="inlineStr">
+      <c r="J19" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">29th july </t>
         </is>
       </c>
-      <c r="J19" s="40" t="n"/>
+      <c r="K19" s="40" t="n"/>
     </row>
     <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="9" t="inlineStr">
+      <c r="A20" s="49" t="n">
+        <v>10</v>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
         <is>
           <t>2026-07-29</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="C20" s="7" t="inlineStr">
         <is>
           <t>Form a central RFI Management system</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t>RFI - Internal</t>
         </is>
       </c>
-      <c r="D20" s="9" t="n">
+      <c r="E20" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="F20" s="7" t="inlineStr">
         <is>
           <t>Documentation</t>
         </is>
       </c>
-      <c r="F20" s="9" t="n"/>
-      <c r="G20" s="18" t="n"/>
-      <c r="H20" s="9" t="inlineStr">
+      <c r="G20" s="9" t="n"/>
+      <c r="H20" s="18" t="n"/>
+      <c r="I20" s="9" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="I20" s="9" t="inlineStr"/>
-      <c r="J20" s="7" t="inlineStr"/>
+      <c r="J20" s="9" t="inlineStr"/>
+      <c r="K20" s="7" t="inlineStr"/>
     </row>
     <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="A21" s="49" t="n">
+        <v>11</v>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="C21" s="8" t="inlineStr">
         <is>
           <t>Brief H&amp;T on fit-out scope and drawings + consolidated info request (substructure, sample drawings, technical data sheets)</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="D21" s="8" t="inlineStr">
         <is>
           <t>Fitout SHD</t>
         </is>
       </c>
-      <c r="D21" s="10" t="n">
+      <c r="E21" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E21" s="8" t="inlineStr">
+      <c r="F21" s="8" t="inlineStr">
         <is>
           <t>Send an email</t>
         </is>
       </c>
-      <c r="F21" s="10" t="n"/>
-      <c r="G21" s="18" t="n"/>
-      <c r="H21" s="10" t="inlineStr">
+      <c r="G21" s="10" t="n"/>
+      <c r="H21" s="18" t="n"/>
+      <c r="I21" s="10" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="I21" s="10" t="inlineStr">
+      <c r="J21" s="10" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="J21" s="8" t="inlineStr">
+      <c r="K21" s="8" t="inlineStr">
         <is>
           <t>Per 29 Jul MoM: one consolidated email, not sequential individual requests. Due today.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="24" customHeight="1">
-      <c r="A22" s="10" t="inlineStr">
+      <c r="A22" s="49" t="n">
+        <v>12</v>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
         <is>
           <t>Finish the AI-created COC and shift to OneDrive to maintain from there</t>
         </is>
       </c>
-      <c r="C22" s="8" t="inlineStr">
+      <c r="D22" s="8" t="inlineStr">
         <is>
           <t>COC Management</t>
         </is>
       </c>
-      <c r="D22" s="10" t="n">
+      <c r="E22" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="F22" s="8" t="inlineStr">
         <is>
           <t>Documentation</t>
         </is>
       </c>
-      <c r="F22" s="10" t="n"/>
-      <c r="G22" s="18" t="n"/>
-      <c r="H22" s="10" t="inlineStr">
+      <c r="G22" s="10" t="n"/>
+      <c r="H22" s="18" t="n"/>
+      <c r="I22" s="10" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="I22" s="10" t="inlineStr"/>
-      <c r="J22" s="8" t="inlineStr"/>
+      <c r="J22" s="10" t="inlineStr"/>
+      <c r="K22" s="8" t="inlineStr"/>
     </row>
     <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="9" t="inlineStr">
+      <c r="A23" s="49" t="n">
+        <v>13</v>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>Finish the Project Calendar and move to OneDrive to maintain from there</t>
         </is>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>WDCO Internal Project Management</t>
         </is>
       </c>
-      <c r="D23" s="9" t="n">
+      <c r="E23" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="F23" s="7" t="inlineStr">
         <is>
           <t>Documentation</t>
         </is>
       </c>
-      <c r="F23" s="9" t="n"/>
-      <c r="G23" s="18" t="n"/>
-      <c r="H23" s="9" t="inlineStr">
+      <c r="G23" s="9" t="n"/>
+      <c r="H23" s="18" t="n"/>
+      <c r="I23" s="9" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="I23" s="9" t="inlineStr"/>
-      <c r="J23" s="7" t="inlineStr">
+      <c r="J23" s="9" t="inlineStr"/>
+      <c r="K23" s="7" t="inlineStr">
         <is>
           <t>Aesthetic alignment only remaining, per Shagun's own 29 Jul note.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="24" customHeight="1">
-      <c r="A24" s="10" t="inlineStr">
+      <c r="A24" s="49" t="n">
+        <v>14</v>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="C24" s="8" t="inlineStr">
         <is>
           <t>Collate feedback on FFE SHD00 to start work on SHD01</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="D24" s="8" t="inlineStr">
         <is>
           <t>FFE SHD</t>
         </is>
       </c>
-      <c r="D24" s="10" t="n">
+      <c r="E24" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="F24" s="8" t="inlineStr">
         <is>
           <t>Documentation</t>
         </is>
       </c>
-      <c r="F24" s="10" t="n"/>
-      <c r="G24" s="18" t="n"/>
-      <c r="H24" s="10" t="inlineStr">
+      <c r="G24" s="10" t="n"/>
+      <c r="H24" s="18" t="n"/>
+      <c r="I24" s="10" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="I24" s="10" t="inlineStr"/>
-      <c r="J24" s="8" t="inlineStr"/>
+      <c r="J24" s="10" t="inlineStr"/>
+      <c r="K24" s="8" t="inlineStr"/>
     </row>
     <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="9" t="inlineStr">
+      <c r="A25" s="49" t="n">
+        <v>15</v>
+      </c>
+      <c r="B25" s="9" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>Fitout Fabrics — banquette fabric sheet — check with suppliers for samples</t>
         </is>
       </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t>Material Package Fitout</t>
         </is>
       </c>
-      <c r="D25" s="9" t="n">
+      <c r="E25" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E25" s="7" t="inlineStr">
+      <c r="F25" s="7" t="inlineStr">
         <is>
           <t>Follow up email</t>
         </is>
       </c>
-      <c r="F25" s="9" t="n"/>
-      <c r="G25" s="18" t="n"/>
-      <c r="H25" s="9" t="inlineStr">
+      <c r="G25" s="9" t="n"/>
+      <c r="H25" s="18" t="n"/>
+      <c r="I25" s="9" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="I25" s="9" t="inlineStr"/>
-      <c r="J25" s="7" t="inlineStr"/>
+      <c r="J25" s="9" t="inlineStr"/>
+      <c r="K25" s="7" t="inlineStr"/>
     </row>
     <row r="26" ht="24" customHeight="1">
-      <c r="A26" s="10" t="inlineStr">
+      <c r="A26" s="49" t="n">
+        <v>16</v>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="B26" s="8" t="inlineStr">
+      <c r="C26" s="8" t="inlineStr">
         <is>
           <t>Create a Google SketchUp model for the project briefing</t>
         </is>
       </c>
-      <c r="C26" s="8" t="inlineStr">
+      <c r="D26" s="8" t="inlineStr">
         <is>
           <t>WDCO Internal Project Management</t>
         </is>
       </c>
-      <c r="D26" s="10" t="n">
+      <c r="E26" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="F26" s="8" t="inlineStr">
         <is>
           <t>Arranging</t>
         </is>
       </c>
-      <c r="F26" s="10" t="n"/>
-      <c r="G26" s="18" t="n"/>
-      <c r="H26" s="10" t="inlineStr">
+      <c r="G26" s="10" t="n"/>
+      <c r="H26" s="18" t="n"/>
+      <c r="I26" s="10" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="I26" s="10" t="inlineStr">
+      <c r="J26" s="10" t="inlineStr">
         <is>
           <t>2026-08-02</t>
         </is>
       </c>
-      <c r="J26" s="8" t="inlineStr">
+      <c r="K26" s="8" t="inlineStr">
         <is>
           <t>Hoped for before Monday's meeting — Type of Task guessed, doesn't cleanly fit the 7 categories.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="9" t="inlineStr">
+      <c r="A27" s="49" t="n">
+        <v>17</v>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="B27" s="7" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>Add fitted-sofa client sample request to fabrication schedule and arrange sample</t>
         </is>
       </c>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>Material Package Fitout</t>
         </is>
       </c>
-      <c r="D27" s="9" t="n">
+      <c r="E27" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E27" s="7" t="inlineStr">
+      <c r="F27" s="7" t="inlineStr">
         <is>
           <t>Arranging</t>
         </is>
       </c>
-      <c r="F27" s="9" t="n"/>
-      <c r="G27" s="18" t="n"/>
-      <c r="H27" s="9" t="inlineStr">
+      <c r="G27" s="9" t="n"/>
+      <c r="H27" s="18" t="n"/>
+      <c r="I27" s="9" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="I27" s="9" t="inlineStr"/>
-      <c r="J27" s="7" t="inlineStr">
+      <c r="J27" s="9" t="inlineStr"/>
+      <c r="K27" s="7" t="inlineStr">
         <is>
           <t>Per 29 Jul MoM.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="24" customHeight="1">
-      <c r="A28" s="10" t="inlineStr">
+      <c r="A28" s="49" t="n">
+        <v>18</v>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="B28" s="8" t="inlineStr">
+      <c r="C28" s="8" t="inlineStr">
         <is>
           <t>Send WDCO project information to the new lighting designer</t>
         </is>
       </c>
-      <c r="C28" s="8" t="inlineStr">
+      <c r="D28" s="8" t="inlineStr">
         <is>
           <t>Communication Management - Client</t>
         </is>
       </c>
-      <c r="D28" s="10" t="n">
+      <c r="E28" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E28" s="8" t="inlineStr">
+      <c r="F28" s="8" t="inlineStr">
         <is>
           <t>Send an email</t>
         </is>
       </c>
-      <c r="F28" s="10" t="n"/>
-      <c r="G28" s="18" t="n"/>
-      <c r="H28" s="10" t="inlineStr">
+      <c r="G28" s="10" t="n"/>
+      <c r="H28" s="18" t="n"/>
+      <c r="I28" s="10" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I28" s="10" t="inlineStr">
+      <c r="J28" s="10" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="J28" s="8" t="inlineStr">
+      <c r="K28" s="8" t="inlineStr">
         <is>
           <t>Introduction email sent 30 Jul. Still need the designer's actual name/email for CONTACT_SHEET.md.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="24" customHeight="1">
-      <c r="A29" s="9" t="inlineStr">
+      <c r="A29" s="49" t="n">
+        <v>19</v>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>Follow up with Victoire on glass sample GL-3A for better specification clarity</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="D29" s="7" t="inlineStr">
         <is>
           <t>Material Package FFE</t>
         </is>
       </c>
-      <c r="D29" s="9" t="n">
+      <c r="E29" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="E29" s="7" t="inlineStr">
+      <c r="F29" s="7" t="inlineStr">
         <is>
           <t>Follow up email</t>
         </is>
       </c>
-      <c r="F29" s="9" t="n"/>
-      <c r="G29" s="18" t="n"/>
-      <c r="H29" s="9" t="inlineStr">
+      <c r="G29" s="9" t="n"/>
+      <c r="H29" s="18" t="n"/>
+      <c r="I29" s="9" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="I29" s="9" t="inlineStr"/>
-      <c r="J29" s="7" t="inlineStr">
+      <c r="J29" s="9" t="inlineStr"/>
+      <c r="K29" s="7" t="inlineStr">
         <is>
           <t>Per 29 Jul MoM.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="24" customHeight="1">
-      <c r="A30" s="10" t="inlineStr">
+      <c r="A30" s="49" t="n">
+        <v>20</v>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="B30" s="8" t="inlineStr">
+      <c r="C30" s="8" t="inlineStr">
         <is>
           <t>Raise an RFI with the lighting designer</t>
         </is>
       </c>
-      <c r="C30" s="8" t="inlineStr">
+      <c r="D30" s="8" t="inlineStr">
         <is>
           <t>RFI - Client</t>
         </is>
       </c>
-      <c r="D30" s="10" t="n">
+      <c r="E30" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E30" s="8" t="inlineStr">
+      <c r="F30" s="8" t="inlineStr">
         <is>
           <t>Send an email</t>
         </is>
       </c>
-      <c r="F30" s="10" t="n"/>
-      <c r="G30" s="18" t="n"/>
-      <c r="H30" s="11" t="inlineStr">
+      <c r="G30" s="10" t="n"/>
+      <c r="H30" s="18" t="n"/>
+      <c r="I30" s="11" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="I30" s="10" t="inlineStr">
+      <c r="J30" s="10" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="J30" s="8" t="inlineStr">
+      <c r="K30" s="8" t="inlineStr">
         <is>
           <t>Email sent 30 Jul referencing the existing FF&amp;E lighting RFI (Sheet 3, 'Lighting / Lighting Equipment Only RFI') — requested equipment details/compliance clarifications from Gisela. Recipient confirmed as the same Gisela Steiger already in CONTACT_SHEET.md, not a new contact. Awaiting her reply; must close by 6 Aug.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="24" customHeight="1">
-      <c r="A31" s="9" t="inlineStr">
+      <c r="A31" s="49" t="n">
+        <v>21</v>
+      </c>
+      <c r="B31" s="9" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="C31" s="7" t="inlineStr">
         <is>
           <t>Follow up with Gisela — structured Fit-out RFI list and workflow</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="D31" s="7" t="inlineStr">
         <is>
           <t>RFI - Client</t>
         </is>
       </c>
-      <c r="D31" s="9" t="n">
+      <c r="E31" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="E31" s="7" t="inlineStr">
+      <c r="F31" s="7" t="inlineStr">
         <is>
           <t>Send an email</t>
         </is>
       </c>
-      <c r="F31" s="9" t="n"/>
-      <c r="G31" s="18" t="n"/>
-      <c r="H31" s="9" t="inlineStr">
+      <c r="G31" s="9" t="n"/>
+      <c r="H31" s="18" t="n"/>
+      <c r="I31" s="9" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="I31" s="9" t="inlineStr">
+      <c r="J31" s="9" t="inlineStr">
         <is>
           <t>2026-08-06</t>
         </is>
       </c>
-      <c r="J31" s="7" t="inlineStr">
+      <c r="K31" s="7" t="inlineStr">
         <is>
           <t>Committed to this in the 30 Jul status email — 'by next week I should be able to share a clearer RFI list and workflow.'</t>
         </is>
       </c>
     </row>
     <row r="32" ht="24" customHeight="1">
-      <c r="A32" s="10" t="inlineStr">
+      <c r="A32" s="49" t="n">
+        <v>22</v>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="B32" s="8" t="inlineStr">
+      <c r="C32" s="8" t="inlineStr">
         <is>
           <t>Create a central RFI tracking system within git</t>
         </is>
       </c>
-      <c r="C32" s="8" t="inlineStr">
+      <c r="D32" s="8" t="inlineStr">
         <is>
           <t>RFI - Internal</t>
         </is>
       </c>
-      <c r="D32" s="10" t="n">
+      <c r="E32" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="E32" s="8" t="inlineStr">
+      <c r="F32" s="8" t="inlineStr">
         <is>
           <t>Documentation</t>
         </is>
       </c>
-      <c r="F32" s="10" t="n"/>
-      <c r="G32" s="18" t="n"/>
-      <c r="H32" s="10" t="inlineStr">
+      <c r="G32" s="10" t="n"/>
+      <c r="H32" s="18" t="n"/>
+      <c r="I32" s="10" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="I32" s="10" t="inlineStr"/>
-      <c r="J32" s="8" t="inlineStr">
+      <c r="J32" s="10" t="inlineStr"/>
+      <c r="K32" s="8" t="inlineStr">
         <is>
           <t>Likely the same initiative as 'Form a central RFI Management system' (29 Jul) — confirm if these should merge into one task.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="24" customHeight="1">
-      <c r="A33" s="46" t="inlineStr">
+      <c r="A33" s="49" t="n">
+        <v>23</v>
+      </c>
+      <c r="B33" s="46" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="B33" s="47" t="inlineStr">
+      <c r="C33" s="47" t="inlineStr">
         <is>
           <t>Prepare agenda for BOQ scope gap meeting (Monday, 3 Aug)</t>
         </is>
       </c>
-      <c r="C33" s="46" t="inlineStr">
+      <c r="D33" s="46" t="inlineStr">
         <is>
           <t>Project Scope</t>
         </is>
       </c>
-      <c r="D33" s="46" t="n">
+      <c r="E33" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="E33" s="47" t="inlineStr">
+      <c r="F33" s="47" t="inlineStr">
         <is>
           <t>Documentation</t>
         </is>
       </c>
-      <c r="F33" s="47" t="inlineStr"/>
       <c r="G33" s="47" t="inlineStr"/>
-      <c r="H33" s="48" t="inlineStr">
+      <c r="H33" s="47" t="inlineStr"/>
+      <c r="I33" s="48" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="I33" s="46" t="inlineStr">
+      <c r="J33" s="46" t="inlineStr">
         <is>
           <t>2026-07-30</t>
         </is>
       </c>
-      <c r="J33" s="47" t="inlineStr">
+      <c r="K33" s="47" t="inlineStr">
         <is>
           <t>Agenda covers: stone arch over wardrobe/fitted sofa, suspended glass light over basin, hardware &amp; bathroom fittings. Stored at meetings/260803_K5M_Meeting_BOQ_Scope_Gap/pre-meeting/agenda.md.</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="24.5" customHeight="1"/>
+    <row r="34" ht="24.5" customHeight="1">
+      <c r="A34" s="46" t="n">
+        <v>24</v>
+      </c>
+      <c r="B34" s="46" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C34" s="47" t="inlineStr">
+        <is>
+          <t>Finish formatting the Project Calendar and Task Tracker to shift both to OneDrive</t>
+        </is>
+      </c>
+      <c r="D34" s="47" t="inlineStr">
+        <is>
+          <t>WDCO Internal Project Management</t>
+        </is>
+      </c>
+      <c r="E34" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="47" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="G34" s="47" t="inlineStr"/>
+      <c r="H34" s="47" t="inlineStr"/>
+      <c r="I34" s="46" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J34" s="46" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="K34" s="47" t="inlineStr">
+        <is>
+          <t>Overlaps with existing rows for the Calendar — this is the combined push to get both files OneDrive-ready today; confirm if those should be marked done/merged once this closes.</t>
+        </is>
+      </c>
+    </row>
     <row r="35" ht="24.5" customHeight="1"/>
     <row r="36" ht="24.5" customHeight="1"/>
     <row r="37" ht="24.5" customHeight="1"/>
@@ -2040,37 +2223,37 @@
     <row r="52" ht="24.5" customHeight="1"/>
     <row r="53" ht="24.5" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A10:J33"/>
+  <autoFilter ref="A10:K34"/>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A2:I2"/>
   </mergeCells>
-  <conditionalFormatting sqref="H11:H32">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
+  <conditionalFormatting sqref="I11:I64">
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="9">
       <formula>"To Do"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="10" operator="equal" dxfId="10">
       <formula>"In Progress"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="5">
+    <cfRule type="cellIs" priority="11" operator="equal" dxfId="11">
       <formula>"Done"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="6">
+    <cfRule type="cellIs" priority="12" operator="equal" dxfId="12">
       <formula>"Stale"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D11:D32">
-    <cfRule type="cellIs" priority="5" operator="equal" dxfId="7">
+  <conditionalFormatting sqref="E11:E64">
+    <cfRule type="cellIs" priority="13" operator="equal" dxfId="13">
       <formula>1</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" dxfId="4">
+    <cfRule type="cellIs" priority="14" operator="equal" dxfId="10">
       <formula>2</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" dxfId="8">
+    <cfRule type="cellIs" priority="15" operator="equal" dxfId="14">
       <formula>3</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="8" operator="equal" dxfId="3">
+    <cfRule type="cellIs" priority="16" operator="equal" dxfId="9">
       <formula>4</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
totalcheck: add security-protocol redaction decision as row 26; mark row 9 (H&T material package agenda) Stale and hide it, superseded by today's meeting
</commit_message>
<xml_diff>
--- a/260730_K5M_Task Tracker.xlsx
+++ b/260730_K5M_Task Tracker.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Task Tracker'!$A$10:$K$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Task Tracker'!$A$10:$K$36</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -1041,7 +1041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1535,7 +1535,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="24" customHeight="1">
+    <row r="19" hidden="1" ht="24" customHeight="1">
       <c r="A19" s="49" t="n">
         <v>9</v>
       </c>
@@ -1566,7 +1566,7 @@
       <c r="H19" s="18" t="n"/>
       <c r="I19" s="10" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Stale</t>
         </is>
       </c>
       <c r="J19" s="23" t="inlineStr">
@@ -1574,7 +1574,11 @@
           <t xml:space="preserve">29th july </t>
         </is>
       </c>
-      <c r="K19" s="40" t="n"/>
+      <c r="K19" s="40" t="inlineStr">
+        <is>
+          <t>Superseded — H&amp;T Material Package review meeting already happened (30 Jul, 10am). Marked Stale + hidden by Woody during #totalcheck.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="24" customHeight="1">
       <c r="A20" s="49" t="n">
@@ -2252,7 +2256,47 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="24.5" customHeight="1"/>
+    <row r="36" ht="24.5" customHeight="1">
+      <c r="A36" s="46" t="n">
+        <v>26</v>
+      </c>
+      <c r="B36" s="46" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="C36" s="47" t="inlineStr">
+        <is>
+          <t>Decide redaction scope for real client/Production Partner names found in README.md, PROJECT_BRIEFING.md, SESSION_START.md, and DAILY_LOG.md (main branch)</t>
+        </is>
+      </c>
+      <c r="D36" s="47" t="inlineStr">
+        <is>
+          <t>WDCO Internal Project Management</t>
+        </is>
+      </c>
+      <c r="E36" s="46" t="n">
+        <v>3</v>
+      </c>
+      <c r="F36" s="47" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="G36" s="47" t="inlineStr"/>
+      <c r="H36" s="47" t="inlineStr"/>
+      <c r="I36" s="46" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J36" s="46" t="inlineStr"/>
+      <c r="K36" s="47" t="inlineStr">
+        <is>
+          <t>Flagged while building HARD_RULES.md — Shagun asked to hold off deciding scope (fix living docs only vs. also rewrite DAILY_LOG history vs. keep Wood Couture as-is). Revisit when ready.</t>
+        </is>
+      </c>
+    </row>
     <row r="37" ht="24.5" customHeight="1"/>
     <row r="38" ht="24.5" customHeight="1"/>
     <row r="39" ht="24.5" customHeight="1"/>
@@ -2271,7 +2315,7 @@
     <row r="52" ht="24.5" customHeight="1"/>
     <row r="53" ht="24.5" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A10:K35"/>
+  <autoFilter ref="A10:K36"/>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A4:B4"/>

</xml_diff>

<commit_message>
Merge duplicate task pairs per Shagun: RFI tracking system (row 10+22) and Calendar/Tracker OneDrive move (row 13+24); mark superseded rows Stale and hide
</commit_message>
<xml_diff>
--- a/260730_K5M_Task Tracker.xlsx
+++ b/260730_K5M_Task Tracker.xlsx
@@ -1591,7 +1591,7 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Form a central RFI Management system</t>
+          <t>Form a central RFI tracking/management system within git</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
@@ -1615,7 +1615,11 @@
         </is>
       </c>
       <c r="J20" s="9" t="inlineStr"/>
-      <c r="K20" s="7" t="inlineStr"/>
+      <c r="K20" s="7" t="inlineStr">
+        <is>
+          <t>Merged with former row 22 (duplicate ask) on 30 Jul per Shagun.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="24" customHeight="1">
       <c r="A21" s="49" t="n">
@@ -1710,7 +1714,7 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Finish the Project Calendar and move to OneDrive to maintain from there</t>
+          <t>Finish formatting the Project Calendar and Task Tracker, and move both to OneDrive to maintain from there</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -1719,7 +1723,7 @@
         </is>
       </c>
       <c r="E23" s="9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
@@ -1733,10 +1737,14 @@
           <t>In Progress</t>
         </is>
       </c>
-      <c r="J23" s="9" t="inlineStr"/>
+      <c r="J23" s="9" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
       <c r="K23" s="7" t="inlineStr">
         <is>
-          <t>Aesthetic alignment only remaining, per Shagun's own 29 Jul note.</t>
+          <t>Merged with former row 24 (duplicate ask) on 30 Jul per Shagun. Aesthetic alignment pass by Shagun, then final push to OneDrive.</t>
         </is>
       </c>
     </row>
@@ -2076,7 +2084,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="24" customHeight="1">
+    <row r="32" hidden="1" ht="24" customHeight="1">
       <c r="A32" s="49" t="n">
         <v>22</v>
       </c>
@@ -2107,13 +2115,13 @@
       <c r="H32" s="18" t="n"/>
       <c r="I32" s="10" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Stale</t>
         </is>
       </c>
       <c r="J32" s="10" t="inlineStr"/>
       <c r="K32" s="8" t="inlineStr">
         <is>
-          <t>Likely the same initiative as 'Form a central RFI Management system' (29 Jul) — confirm if these should merge into one task.</t>
+          <t>Merged into row 10 (duplicate) — marked Stale + hidden by Woody, 30 Jul.</t>
         </is>
       </c>
     </row>
@@ -2162,7 +2170,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="24.5" customHeight="1">
+    <row r="34" hidden="1" ht="24.5" customHeight="1">
       <c r="A34" s="46" t="n">
         <v>24</v>
       </c>
@@ -2193,7 +2201,7 @@
       <c r="H34" s="47" t="inlineStr"/>
       <c r="I34" s="46" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Stale</t>
         </is>
       </c>
       <c r="J34" s="46" t="inlineStr">
@@ -2203,7 +2211,7 @@
       </c>
       <c r="K34" s="47" t="inlineStr">
         <is>
-          <t>Overlaps with existing rows for the Calendar — this is the combined push to get both files OneDrive-ready today; confirm if those should be marked done/merged once this closes.</t>
+          <t>Merged into row 13 (duplicate) — marked Stale + hidden by Woody, 30 Jul.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
newtask: align product codes across trackers (row 27), raised after CHA-RT-01/CHA-ST-02 mismatch
</commit_message>
<xml_diff>
--- a/260730_K5M_Task Tracker.xlsx
+++ b/260730_K5M_Task Tracker.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Task Tracker'!$A$10:$K$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Task Tracker'!$A$10:$K$37</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -1041,7 +1041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2305,7 +2305,47 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="24.5" customHeight="1"/>
+    <row r="37" ht="24.5" customHeight="1">
+      <c r="A37" s="46" t="n">
+        <v>27</v>
+      </c>
+      <c r="B37" s="46" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C37" s="47" t="inlineStr">
+        <is>
+          <t>Align all product codes across trackers (Material Package, COC Master Scope, client-facing documents) — especially client-facing product codes</t>
+        </is>
+      </c>
+      <c r="D37" s="47" t="inlineStr">
+        <is>
+          <t>COC Management</t>
+        </is>
+      </c>
+      <c r="E37" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" s="47" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="G37" s="47" t="inlineStr"/>
+      <c r="H37" s="47" t="inlineStr"/>
+      <c r="I37" s="46" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J37" s="46" t="inlineStr"/>
+      <c r="K37" s="47" t="inlineStr">
+        <is>
+          <t>Raised after finding K5M-T1B1-CHA-RT-01 in the Material Package with no match in the COC Master Scope — traced to the Small Round Table (CG03), correctly coded K5M-T1B1-CHA-ST-02 in the COC. Gap between manual entries and Woody-maintained trackers. Umbrella Task/Priority guessed, flag for correction.</t>
+        </is>
+      </c>
+    </row>
     <row r="38" ht="24.5" customHeight="1"/>
     <row r="39" ht="24.5" customHeight="1"/>
     <row r="40" ht="24.5" customHeight="1"/>
@@ -2323,7 +2363,7 @@
     <row r="52" ht="24.5" customHeight="1"/>
     <row r="53" ht="24.5" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A10:K36"/>
+  <autoFilter ref="A10:K37"/>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A4:B4"/>

</xml_diff>

<commit_message>
newtask: decide base project scope file(s), row 28 -- pending decision to become a hard rule
</commit_message>
<xml_diff>
--- a/260730_K5M_Task Tracker.xlsx
+++ b/260730_K5M_Task Tracker.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Task Tracker'!$A$10:$K$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Task Tracker'!$A$10:$K$38</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -1041,7 +1041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2346,7 +2346,47 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="24.5" customHeight="1"/>
+    <row r="38" ht="24.5" customHeight="1">
+      <c r="A38" s="46" t="n">
+        <v>28</v>
+      </c>
+      <c r="B38" s="46" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C38" s="47" t="inlineStr">
+        <is>
+          <t>Decide and inform Woody which project scope file(s) will be the base/authoritative source for all documents going forward</t>
+        </is>
+      </c>
+      <c r="D38" s="47" t="inlineStr">
+        <is>
+          <t>COC Management</t>
+        </is>
+      </c>
+      <c r="E38" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" s="47" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="G38" s="47" t="inlineStr"/>
+      <c r="H38" s="47" t="inlineStr"/>
+      <c r="I38" s="46" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J38" s="46" t="inlineStr"/>
+      <c r="K38" s="47" t="inlineStr">
+        <is>
+          <t>Directly related to row 27 (product code alignment). Once decided, this becomes a hard rule — add to HARD_RULES.md (main branch) once confirmed.</t>
+        </is>
+      </c>
+    </row>
     <row r="39" ht="24.5" customHeight="1"/>
     <row r="40" ht="24.5" customHeight="1"/>
     <row r="41" ht="24.5" customHeight="1"/>
@@ -2363,7 +2403,7 @@
     <row r="52" ht="24.5" customHeight="1"/>
     <row r="53" ht="24.5" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A10:K37"/>
+  <autoFilter ref="A10:K38"/>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A4:B4"/>

</xml_diff>

<commit_message>
Update rows 27/28: FFE scope codes aligned, canonical FFE scope file confirmed; Fitout still pending
</commit_message>
<xml_diff>
--- a/260730_K5M_Task Tracker.xlsx
+++ b/260730_K5M_Task Tracker.xlsx
@@ -2336,13 +2336,13 @@
       <c r="H37" s="47" t="inlineStr"/>
       <c r="I37" s="46" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J37" s="46" t="inlineStr"/>
       <c r="K37" s="47" t="inlineStr">
         <is>
-          <t>Raised after finding K5M-T1B1-CHA-RT-01 in the Material Package with no match in the COC Master Scope — traced to the Small Round Table (CG03), correctly coded K5M-T1B1-CHA-ST-02 in the COC. Gap between manual entries and Woody-maintained trackers. Umbrella Task/Priority guessed, flag for correction.</t>
+          <t>FFE scope codes now aligned (CH→CHA fixed 31 Jul in the canonical Master SKU List). Material Package’s own CHA-RT-01 error still unfixed there (Shagun deferred that edit). Fitout scope not yet confirmed — expected next week; recheck fitout codes once that lands.</t>
         </is>
       </c>
     </row>
@@ -2377,13 +2377,13 @@
       <c r="H38" s="47" t="inlineStr"/>
       <c r="I38" s="46" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J38" s="46" t="inlineStr"/>
       <c r="K38" s="47" t="inlineStr">
         <is>
-          <t>Directly related to row 27 (product code alignment). Once decided, this becomes a hard rule — add to HARD_RULES.md (main branch) once confirmed.</t>
+          <t>FFE resolved 31 Jul — holy grail file confirmed: 260724_WDCOK5M_FFE_Master SKU List.xlsx (OneDrive, 00_SHARED/Project Scope). Now added to HARD_RULES.md. Fitout base scope file still pending — Shagun expects to confirm next week.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
File H&T Material Package MOM (31 Jul) into meeting folder; log as row 29 in Task Tracker
</commit_message>
<xml_diff>
--- a/260730_K5M_Task Tracker.xlsx
+++ b/260730_K5M_Task Tracker.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Task Tracker'!$A$10:$K$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Task Tracker'!$A$10:$K$39</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -1041,7 +1041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L38"/>
+  <dimension ref="A1:L39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2387,7 +2387,51 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="24.5" customHeight="1"/>
+    <row r="39" ht="24.5" customHeight="1">
+      <c r="A39" s="46" t="n">
+        <v>29</v>
+      </c>
+      <c r="B39" s="46" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="C39" s="47" t="inlineStr">
+        <is>
+          <t>File H&amp;T Meeting Minutes (MOM, 31 Jul — material package development) into the repo meeting folder</t>
+        </is>
+      </c>
+      <c r="D39" s="47" t="inlineStr">
+        <is>
+          <t>Communication Management - Production Partner</t>
+        </is>
+      </c>
+      <c r="E39" s="46" t="n">
+        <v>2</v>
+      </c>
+      <c r="F39" s="47" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="G39" s="47" t="inlineStr"/>
+      <c r="H39" s="47" t="inlineStr"/>
+      <c r="I39" s="46" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="J39" s="46" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="K39" s="47" t="inlineStr">
+        <is>
+          <t>Filed at meetings/260731_K5M_Meeting_H&amp;T_Material_Package/minutes/. Not a duplicate of the #projectdevelopment Dev Log entries — those capture the narrative, this is the source document.</t>
+        </is>
+      </c>
+    </row>
     <row r="40" ht="24.5" customHeight="1"/>
     <row r="41" ht="24.5" customHeight="1"/>
     <row r="42" ht="24.5" customHeight="1"/>
@@ -2403,7 +2447,7 @@
     <row r="52" ht="24.5" customHeight="1"/>
     <row r="53" ht="24.5" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A10:K38"/>
+  <autoFilter ref="A10:K39"/>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A4:B4"/>

</xml_diff>

<commit_message>
totalcheck: fix row 4 due-date discrepancy (Aug 5, not Sep 5), update row 15 Fitout fabrics to In Progress
</commit_message>
<xml_diff>
--- a/260730_K5M_Task Tracker.xlsx
+++ b/260730_K5M_Task Tracker.xlsx
@@ -1363,9 +1363,13 @@
         </is>
       </c>
       <c r="J14" s="52" t="n">
-        <v>46270</v>
-      </c>
-      <c r="K14" s="51" t="inlineStr"/>
+        <v>46239</v>
+      </c>
+      <c r="K14" s="51" t="inlineStr">
+        <is>
+          <t>Due date corrected 31 Jul (was 05/09/2026, a month off) — matches the 5 Aug Calendar milestone and the urgency flagged in this week's risk-mitigation note: implementation cannot start until this is sent.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="24" customHeight="1" thickBot="1">
       <c r="A15" s="49" t="n">
@@ -1816,11 +1820,15 @@
       <c r="H25" s="18" t="n"/>
       <c r="I25" s="9" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J25" s="9" t="inlineStr"/>
-      <c r="K25" s="7" t="inlineStr"/>
+      <c r="K25" s="7" t="inlineStr">
+        <is>
+          <t>Per 31 Jul H&amp;T meeting — Fit-out fabrics partially researched online, findings updated in the Excel sheet and fabric folder shared.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="49" t="n">

</xml_diff>

<commit_message>
Fix column widths misaligned with headers since the S.No. column insert (Task/Umbrella Task/Note were badly cramped, Date Raised/Due Date oversized)
</commit_message>
<xml_diff>
--- a/260730_K5M_Task Tracker.xlsx
+++ b/260730_K5M_Task Tracker.xlsx
@@ -1045,15 +1045,16 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="62" customWidth="1" min="2" max="2"/>
-    <col width="31" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="52" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">

</xml_diff>

<commit_message>
totalcheck: update row 12 note to reflect COC full-rebuild decision
</commit_message>
<xml_diff>
--- a/260730_K5M_Task Tracker.xlsx
+++ b/260730_K5M_Task Tracker.xlsx
@@ -1706,7 +1706,11 @@
         </is>
       </c>
       <c r="J22" s="10" t="inlineStr"/>
-      <c r="K22" s="8" t="inlineStr"/>
+      <c r="K22" s="8" t="inlineStr">
+        <is>
+          <t>Decided 3 Aug: full rebuild from scratch, once underlying data is fully verified/clean, rather than patching the 28 July v1. Freeze panes removed, Data tab rebuilt from canonical scope, and Hard Material partially updated as interim steps — but the ground-up rebuild is still the plan.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="49" t="n">

</xml_diff>

<commit_message>
Log 4 Aug meeting with Claire: update rows 2/3/11, add 8 new tasks (metal samples, drawings, compliance, BOQ recheck, substructure, site visit, SHD01, Resti connect)
</commit_message>
<xml_diff>
--- a/260730_K5M_Task Tracker.xlsx
+++ b/260730_K5M_Task Tracker.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Task Tracker'!$A$10:$K$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Task Tracker'!$A$10:$K$47</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -1041,7 +1041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1288,7 +1288,7 @@
       <c r="J12" s="10" t="inlineStr"/>
       <c r="K12" s="8" t="inlineStr">
         <is>
-          <t>Per 29 Jul MoM — explicitly flagged High priority, must not slip.</t>
+          <t>Reinforced in 4 Aug meeting with Claire — align presentation/delivery method with internal guidelines, then use Khamille's guidance to prepare a complete sample presentation for H&amp;T.</t>
         </is>
       </c>
     </row>
@@ -1323,13 +1323,13 @@
       <c r="H13" s="18" t="n"/>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J13" s="9" t="inlineStr"/>
       <c r="K13" s="7" t="inlineStr">
         <is>
-          <t>Not explicitly closed by the 29 Jul MoM — confirm still open.</t>
+          <t>Resolved in 4 Aug meeting with Claire — agreed to ask Adil's site team to confirm what substructure work/info already exists, then start H&amp;T communication (see row 4 and new row below).</t>
         </is>
       </c>
     </row>
@@ -1667,7 +1667,7 @@
       </c>
       <c r="K21" s="8" t="inlineStr">
         <is>
-          <t>Per 29 Jul MoM: one consolidated email, not sequential individual requests. Due today.</t>
+          <t>Per 29 Jul MoM: one consolidated email, not sequential individual requests. Reinforced in 4 Aug meeting with Claire — start H&amp;T comms on fit-out scope ASAP, share available info once site team responds, request any additional H&amp;T needs immediately.</t>
         </is>
       </c>
     </row>
@@ -2445,14 +2445,370 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="24.5" customHeight="1"/>
-    <row r="41" ht="24.5" customHeight="1"/>
-    <row r="42" ht="24.5" customHeight="1"/>
-    <row r="43" ht="24.5" customHeight="1"/>
-    <row r="44" ht="24.5" customHeight="1"/>
-    <row r="45" ht="24.5" customHeight="1"/>
-    <row r="46" ht="24.5" customHeight="1"/>
-    <row r="47" ht="24.5" customHeight="1"/>
+    <row r="40" ht="24.5" customHeight="1">
+      <c r="A40" s="46" t="n">
+        <v>30</v>
+      </c>
+      <c r="B40" s="46" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="C40" s="47" t="inlineStr">
+        <is>
+          <t>Ask H&amp;T (China team) to begin developing first metal-sample finishes based on client reference images</t>
+        </is>
+      </c>
+      <c r="D40" s="47" t="inlineStr">
+        <is>
+          <t>Material Package FFE</t>
+        </is>
+      </c>
+      <c r="E40" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" s="47" t="inlineStr">
+        <is>
+          <t>Send an email</t>
+        </is>
+      </c>
+      <c r="G40" s="47" t="inlineStr">
+        <is>
+          <t>H&amp;T</t>
+        </is>
+      </c>
+      <c r="H40" s="47" t="n"/>
+      <c r="I40" s="46" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J40" s="46" t="n"/>
+      <c r="K40" s="47" t="inlineStr">
+        <is>
+          <t>Per 4 Aug meeting with Claire: Paris design team clarified 3 coating finishes look similar but are different codes based on metal nature — doesn't align with VE. Agreed to proceed via H&amp;T China team using client visual references rather than resolving the code discrepancy first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="24.5" customHeight="1">
+      <c r="A41" s="46" t="n">
+        <v>31</v>
+      </c>
+      <c r="B41" s="46" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="C41" s="47" t="inlineStr">
+        <is>
+          <t>Proceed with Ariel for required fit-out drawing updates; copy Resti</t>
+        </is>
+      </c>
+      <c r="D41" s="47" t="inlineStr">
+        <is>
+          <t>Fitout SHD</t>
+        </is>
+      </c>
+      <c r="E41" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" s="47" t="inlineStr">
+        <is>
+          <t>Send an email</t>
+        </is>
+      </c>
+      <c r="G41" s="47" t="inlineStr">
+        <is>
+          <t>Ariel</t>
+        </is>
+      </c>
+      <c r="H41" s="47" t="inlineStr">
+        <is>
+          <t>Resti</t>
+        </is>
+      </c>
+      <c r="I41" s="46" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J41" s="46" t="n"/>
+      <c r="K41" s="47" t="inlineStr">
+        <is>
+          <t>Per 4 Aug meeting with Claire — fit-out drawings must be updated before scope can float further. Resti (Head of Engineering, joined this week) copied to stay informed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="24.5" customHeight="1">
+      <c r="A42" s="46" t="n">
+        <v>32</v>
+      </c>
+      <c r="B42" s="46" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="C42" s="47" t="inlineStr">
+        <is>
+          <t>Request compliance sheets/certificates from Abdellatif Menbar (client) — hardware, bathroom fittings, electrical, stone anti-slip certification, foam, and any other regulated/specified materials</t>
+        </is>
+      </c>
+      <c r="D42" s="47" t="inlineStr">
+        <is>
+          <t>Compliance Collection</t>
+        </is>
+      </c>
+      <c r="E42" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" s="47" t="inlineStr">
+        <is>
+          <t>Send an email</t>
+        </is>
+      </c>
+      <c r="G42" s="47" t="inlineStr">
+        <is>
+          <t>Abdellatif Menbar</t>
+        </is>
+      </c>
+      <c r="H42" s="47" t="n"/>
+      <c r="I42" s="46" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J42" s="46" t="n"/>
+      <c r="K42" s="47" t="inlineStr">
+        <is>
+          <t>Per 4 Aug meeting with Claire. Share the Hyatt reference sheet found online; confirm whether any additional documents/formats are required.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="24.5" customHeight="1">
+      <c r="A43" s="46" t="n">
+        <v>33</v>
+      </c>
+      <c r="B43" s="46" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="C43" s="47" t="inlineStr">
+        <is>
+          <t>Ask Resti to recheck stone arch measurements/quantities; communicate scope gaps and changes since kick-off transparently to stakeholders</t>
+        </is>
+      </c>
+      <c r="D43" s="47" t="inlineStr">
+        <is>
+          <t>Project Scope</t>
+        </is>
+      </c>
+      <c r="E43" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" s="47" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="G43" s="47" t="inlineStr">
+        <is>
+          <t>Resti</t>
+        </is>
+      </c>
+      <c r="H43" s="47" t="n"/>
+      <c r="I43" s="46" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J43" s="46" t="n"/>
+      <c r="K43" s="47" t="inlineStr">
+        <is>
+          <t>Per 4 Aug meeting with Claire — directly overlaps with the stone arch BOQ scope gap study already done and saved at meetings/260803_K5M_Meeting_BOQ_Scope_Gap/post-meeting/Fit-out BOQ Scope Gap/stone_arch_findings.md. Resti's recheck should reference that file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="24.5" customHeight="1">
+      <c r="A44" s="46" t="n">
+        <v>34</v>
+      </c>
+      <c r="B44" s="46" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="C44" s="47" t="inlineStr">
+        <is>
+          <t>Ask Adil's site team to confirm what substructure work/information has already been prepared</t>
+        </is>
+      </c>
+      <c r="D44" s="47" t="inlineStr">
+        <is>
+          <t>Fitout SHD</t>
+        </is>
+      </c>
+      <c r="E44" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" s="47" t="inlineStr">
+        <is>
+          <t>Send an email</t>
+        </is>
+      </c>
+      <c r="G44" s="47" t="inlineStr">
+        <is>
+          <t>Adil</t>
+        </is>
+      </c>
+      <c r="H44" s="47" t="n"/>
+      <c r="I44" s="46" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J44" s="46" t="n"/>
+      <c r="K44" s="47" t="inlineStr">
+        <is>
+          <t>Per 4 Aug meeting with Claire — substructure info is critical for fit-out drawings, BOQ, supplier scope, and sample development. Share available details with H&amp;T once site team's input received (see row 11).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="24.5" customHeight="1">
+      <c r="A45" s="46" t="n">
+        <v>35</v>
+      </c>
+      <c r="B45" s="46" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="C45" s="47" t="inlineStr">
+        <is>
+          <t>Plan the 31 Aug–1 Sep site visit — start comms with H&amp;T on dates, prepare/circulate agenda (objectives, attendees, sample review, site activities, deliverables, responsibilities, timings); ask Abdellatif Menbar/Adil for site-access permits, accommodation, and site location/Maps link</t>
+        </is>
+      </c>
+      <c r="D45" s="47" t="inlineStr">
+        <is>
+          <t>Site Survey Planning</t>
+        </is>
+      </c>
+      <c r="E45" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F45" s="47" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="G45" s="47" t="inlineStr">
+        <is>
+          <t>H&amp;T</t>
+        </is>
+      </c>
+      <c r="H45" s="47" t="n"/>
+      <c r="I45" s="46" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J45" s="46" t="n"/>
+      <c r="K45" s="47" t="inlineStr">
+        <is>
+          <t>Per 4 Aug meeting with Claire — decided today to extend this to a 2-day effort (was previously a single 31 Aug entry). Calendar Hard Milestone updated accordingly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="24.5" customHeight="1">
+      <c r="A46" s="46" t="n">
+        <v>36</v>
+      </c>
+      <c r="B46" s="46" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="C46" s="47" t="inlineStr">
+        <is>
+          <t>Schedule and prepare for the K5M FFE SHD01 review meeting (5 Aug, 10:30am)</t>
+        </is>
+      </c>
+      <c r="D46" s="47" t="inlineStr">
+        <is>
+          <t>FFE SHD</t>
+        </is>
+      </c>
+      <c r="E46" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" s="47" t="inlineStr">
+        <is>
+          <t>Meeting online</t>
+        </is>
+      </c>
+      <c r="G46" s="47" t="n"/>
+      <c r="H46" s="47" t="n"/>
+      <c r="I46" s="46" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J46" s="46" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="K46" s="47" t="inlineStr">
+        <is>
+          <t>Per 4 Aug meeting with Claire. Ensure consolidated feedback ready before the meeting; prepare/circulate latest drawings. The Shop Drawing Tracker (once built) will serve as the meeting agenda — no separate agenda doc planned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="24.5" customHeight="1">
+      <c r="A47" s="46" t="n">
+        <v>37</v>
+      </c>
+      <c r="B47" s="46" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="C47" s="47" t="inlineStr">
+        <is>
+          <t>Connect with Resti as soon as possible to flag current K5M technical support needs</t>
+        </is>
+      </c>
+      <c r="D47" s="47" t="inlineStr">
+        <is>
+          <t>WDCO Internal Project Management</t>
+        </is>
+      </c>
+      <c r="E47" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" s="47" t="inlineStr">
+        <is>
+          <t>Meeting online</t>
+        </is>
+      </c>
+      <c r="G47" s="47" t="inlineStr">
+        <is>
+          <t>Resti</t>
+        </is>
+      </c>
+      <c r="H47" s="47" t="n"/>
+      <c r="I47" s="46" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J47" s="46" t="n"/>
+      <c r="K47" s="47" t="inlineStr">
+        <is>
+          <t>Resti is the new Head of Engineering (joined 2026-08-04) — technical point of reference for shop drawings/engineering support across all projects, working with Tharusha (draftsman). Per his introduction: connect early so he can prioritize.</t>
+        </is>
+      </c>
+    </row>
     <row r="48" ht="24.5" customHeight="1"/>
     <row r="49" ht="24.5" customHeight="1"/>
     <row r="50" ht="24.5" customHeight="1"/>
@@ -2460,7 +2816,7 @@
     <row r="52" ht="24.5" customHeight="1"/>
     <row r="53" ht="24.5" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A10:K39"/>
+  <autoFilter ref="A10:K47"/>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A4:B4"/>

</xml_diff>

<commit_message>
Log 3 Aug BOQ gap meeting decisions + status updates (Resti, Abdellatif, SHD01); add Logistics umbrella task
</commit_message>
<xml_diff>
--- a/260730_K5M_Task Tracker.xlsx
+++ b/260730_K5M_Task Tracker.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Task Tracker'!$A$10:$K$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Task Tracker'!$A$10:$K$56</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -17,7 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  </numFmts>
   <fonts count="16">
     <font>
       <name val="Calibri"/>
@@ -379,7 +381,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -533,6 +535,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="15" fillId="6" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="15" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1041,7 +1046,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1360,7 +1365,7 @@
       <c r="H14" s="47" t="inlineStr"/>
       <c r="I14" s="50" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="J14" s="52" t="n">
@@ -1368,7 +1373,7 @@
       </c>
       <c r="K14" s="51" t="inlineStr">
         <is>
-          <t>Due date corrected 31 Jul (was 05/09/2026, a month off) — matches the 5 Aug Calendar milestone and the urgency flagged in this week's risk-mitigation note: implementation cannot start until this is sent.</t>
+          <t>Due date corrected 31 Jul (was 05/09/2026, a month off) — matches the 5 Aug Calendar milestone and the urgency flagged in this week's risk-mitigation note: implementation cannot start until this is sent. Sent per Claire's 4 Aug direction; further discussion ongoing with Abdellatif Menbar via email — awaiting outcome (per 6 Aug update).</t>
         </is>
       </c>
     </row>
@@ -2574,13 +2579,15 @@
       <c r="H42" s="47" t="n"/>
       <c r="I42" s="46" t="inlineStr">
         <is>
-          <t>To Do</t>
-        </is>
-      </c>
-      <c r="J42" s="46" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J42" s="53" t="n">
+        <v>46244</v>
+      </c>
       <c r="K42" s="47" t="inlineStr">
         <is>
-          <t>Per 4 Aug meeting with Claire. Share the Hyatt reference sheet found online; confirm whether any additional documents/formats are required.</t>
+          <t>Per 4 Aug meeting with Claire. Share the Hyatt reference sheet found online; confirm whether any additional documents/formats are required. Target close 10 Aug (per 3 Aug BOQ gap meeting decision).</t>
         </is>
       </c>
     </row>
@@ -2619,13 +2626,13 @@
       <c r="H43" s="47" t="n"/>
       <c r="I43" s="46" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J43" s="46" t="n"/>
       <c r="K43" s="47" t="inlineStr">
         <is>
-          <t>Per 4 Aug meeting with Claire — directly overlaps with the stone arch BOQ scope gap study already done and saved at meetings/260803_K5M_Meeting_BOQ_Scope_Gap/post-meeting/Fit-out BOQ Scope Gap/stone_arch_findings.md. Resti's recheck should reference that file.</t>
+          <t>Per 4 Aug meeting with Claire — directly overlaps with the stone arch BOQ scope gap study already done and saved at meetings/260803_K5M_Meeting_BOQ_Scope_Gap/post-meeting/Fit-out BOQ Scope Gap/stone_arch_findings.md. Resti's recheck should reference that file. Resti completed the calculation (per 6 Aug update) — being incorporated into a clear write-up, see new row below.</t>
         </is>
       </c>
     </row>
@@ -2715,7 +2722,7 @@
       <c r="J45" s="46" t="n"/>
       <c r="K45" s="47" t="inlineStr">
         <is>
-          <t>Per 4 Aug meeting with Claire — decided today to extend this to a 2-day effort (was previously a single 31 Aug entry). Calendar Hard Milestone updated accordingly.</t>
+          <t>Per 4 Aug meeting with Claire — decided today to extend this to a 2-day effort (was previously a single 31 Aug entry). Calendar Hard Milestone updated accordingly. Site visit timing under ambiguity as of the 3 Aug BOQ gap meeting — regardless, need white-box photos ready and a post-site-survey deliverable prepared.</t>
         </is>
       </c>
     </row>
@@ -2750,7 +2757,7 @@
       <c r="H46" s="47" t="n"/>
       <c r="I46" s="46" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J46" s="46" t="inlineStr">
@@ -2760,7 +2767,7 @@
       </c>
       <c r="K46" s="47" t="inlineStr">
         <is>
-          <t>Per 4 Aug meeting with Claire. Ensure consolidated feedback ready before the meeting; prepare/circulate latest drawings. The Shop Drawing Tracker (once built) will serve as the meeting agenda — no separate agenda doc planned.</t>
+          <t>Per 4 Aug meeting with Claire. Ensure consolidated feedback ready before the meeting; prepare/circulate latest drawings. The Shop Drawing Tracker (once built) will serve as the meeting agenda — no separate agenda doc planned. Meeting held 5 Aug as scheduled. MOM to follow — see new row below; content still pending from Shagun as of 6 Aug.</t>
         </is>
       </c>
     </row>
@@ -2799,24 +2806,417 @@
       <c r="H47" s="47" t="n"/>
       <c r="I47" s="46" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J47" s="46" t="n"/>
       <c r="K47" s="47" t="inlineStr">
         <is>
-          <t>Resti is the new Head of Engineering (joined 2026-08-04) — technical point of reference for shop drawings/engineering support across all projects, working with Tharusha (draftsman). Per his introduction: connect early so he can prioritize.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="24.5" customHeight="1"/>
-    <row r="49" ht="24.5" customHeight="1"/>
-    <row r="50" ht="24.5" customHeight="1"/>
-    <row r="51" ht="24.5" customHeight="1"/>
-    <row r="52" ht="24.5" customHeight="1"/>
-    <row r="53" ht="24.5" customHeight="1"/>
+          <t>Resti is the new Head of Engineering (joined 2026-08-04) — technical point of reference for shop drawings/engineering support across all projects, working with Tharusha (draftsman). Per his introduction: connect early so he can prioritize. Connected — Resti has already completed the stone arch BOQ gap calculation requested (see new row below).</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="24.5" customHeight="1">
+      <c r="A48" s="46" t="n">
+        <v>38</v>
+      </c>
+      <c r="B48" s="46" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="C48" s="47" t="inlineStr">
+        <is>
+          <t>Clearly document Resti's completed stone arch BOQ gap calculation and incorporate it into the existing scope-gap findings</t>
+        </is>
+      </c>
+      <c r="D48" s="47" t="inlineStr">
+        <is>
+          <t>Project Scope</t>
+        </is>
+      </c>
+      <c r="E48" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" s="47" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="G48" s="47" t="inlineStr">
+        <is>
+          <t>Resti</t>
+        </is>
+      </c>
+      <c r="H48" s="47" t="n"/>
+      <c r="I48" s="46" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J48" s="46" t="n"/>
+      <c r="K48" s="47" t="inlineStr">
+        <is>
+          <t>Per 3 Aug BOQ gap meeting decision (a). Resti's raw calculation is complete (see row above) — this is writing it up clearly. References meetings/260803_K5M_Meeting_BOQ_Scope_Gap/post-meeting/Fit-out BOQ Scope Gap/stone_arch_findings.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="24.5" customHeight="1">
+      <c r="A49" s="46" t="n">
+        <v>39</v>
+      </c>
+      <c r="B49" s="46" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="C49" s="47" t="inlineStr">
+        <is>
+          <t>Draft and send an email covering all BOQ changes (the gap, the difference) to Filippo Sona to handle from there</t>
+        </is>
+      </c>
+      <c r="D49" s="47" t="inlineStr">
+        <is>
+          <t>Communication Management - Internal</t>
+        </is>
+      </c>
+      <c r="E49" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" s="47" t="inlineStr">
+        <is>
+          <t>Send an email</t>
+        </is>
+      </c>
+      <c r="G49" s="47" t="inlineStr">
+        <is>
+          <t>Filippo Sona</t>
+        </is>
+      </c>
+      <c r="H49" s="47" t="n"/>
+      <c r="I49" s="46" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J49" s="46" t="n"/>
+      <c r="K49" s="47" t="inlineStr">
+        <is>
+          <t>Per 3 Aug BOQ gap meeting decision (b). Filippo Sona is WDCO's co-founder and main partner — internal, not client-facing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="24.5" customHeight="1">
+      <c r="A50" s="46" t="n">
+        <v>40</v>
+      </c>
+      <c r="B50" s="46" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="C50" s="47" t="inlineStr">
+        <is>
+          <t>Email Maria for container requirements so the container can be scheduled right away</t>
+        </is>
+      </c>
+      <c r="D50" s="47" t="inlineStr">
+        <is>
+          <t>Logistics</t>
+        </is>
+      </c>
+      <c r="E50" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" s="47" t="inlineStr">
+        <is>
+          <t>Send an email</t>
+        </is>
+      </c>
+      <c r="G50" s="47" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="H50" s="47" t="n"/>
+      <c r="I50" s="46" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J50" s="46" t="n"/>
+      <c r="K50" s="47" t="inlineStr">
+        <is>
+          <t>Per 3 Aug BOQ gap meeting decision (c). Maria is WDCO's logistics personnel, handling container booking etc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="24.5" customHeight="1">
+      <c r="A51" s="46" t="n">
+        <v>41</v>
+      </c>
+      <c r="B51" s="46" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="C51" s="47" t="inlineStr">
+        <is>
+          <t>Build a new Fitout Scope document — clearly defining everything, with a "Doubts" section for anything removable/uncertain</t>
+        </is>
+      </c>
+      <c r="D51" s="47" t="inlineStr">
+        <is>
+          <t>Project Scope</t>
+        </is>
+      </c>
+      <c r="E51" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F51" s="47" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="G51" s="47" t="n"/>
+      <c r="H51" s="47" t="n"/>
+      <c r="I51" s="46" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J51" s="46" t="n"/>
+      <c r="K51" s="47" t="inlineStr">
+        <is>
+          <t>Per 3 Aug BOQ gap meeting decision (d). This resolves Hard Rule 14's long-pending Fitout base-scope file once built — update that rule once done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="24.5" customHeight="1">
+      <c r="A52" s="46" t="n">
+        <v>42</v>
+      </c>
+      <c r="B52" s="46" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="C52" s="47" t="inlineStr">
+        <is>
+          <t>Schedule a fitout scope meeting with H&amp;T ASAP</t>
+        </is>
+      </c>
+      <c r="D52" s="47" t="inlineStr">
+        <is>
+          <t>Fitout SHD</t>
+        </is>
+      </c>
+      <c r="E52" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F52" s="47" t="inlineStr">
+        <is>
+          <t>Meeting online</t>
+        </is>
+      </c>
+      <c r="G52" s="47" t="inlineStr">
+        <is>
+          <t>H&amp;T</t>
+        </is>
+      </c>
+      <c r="H52" s="47" t="n"/>
+      <c r="I52" s="46" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J52" s="46" t="n"/>
+      <c r="K52" s="47" t="inlineStr">
+        <is>
+          <t>Per 3 Aug BOQ gap meeting decision (e).</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="24.5" customHeight="1">
+      <c r="A53" s="46" t="n">
+        <v>43</v>
+      </c>
+      <c r="B53" s="46" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="C53" s="47" t="inlineStr">
+        <is>
+          <t>Confirm with Ariel which fitout drawings are shareable</t>
+        </is>
+      </c>
+      <c r="D53" s="47" t="inlineStr">
+        <is>
+          <t>Fitout SHD</t>
+        </is>
+      </c>
+      <c r="E53" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" s="47" t="inlineStr">
+        <is>
+          <t>Follow up email</t>
+        </is>
+      </c>
+      <c r="G53" s="47" t="inlineStr">
+        <is>
+          <t>Ariel</t>
+        </is>
+      </c>
+      <c r="H53" s="47" t="n"/>
+      <c r="I53" s="46" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J53" s="53" t="n">
+        <v>46241</v>
+      </c>
+      <c r="K53" s="47" t="inlineStr">
+        <is>
+          <t>Per 3 Aug BOQ gap meeting decision (f). Deadline of 7 Aug confirmed by Ariel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="46" t="n">
+        <v>44</v>
+      </c>
+      <c r="B54" s="46" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="C54" s="47" t="inlineStr">
+        <is>
+          <t>Send MOM from the internal FFE Shop Drawing (SHD01) review meeting held 5 Aug</t>
+        </is>
+      </c>
+      <c r="D54" s="47" t="inlineStr">
+        <is>
+          <t>FFE SHD</t>
+        </is>
+      </c>
+      <c r="E54" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" s="47" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="G54" s="47" t="n"/>
+      <c r="H54" s="47" t="n"/>
+      <c r="I54" s="46" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J54" s="53" t="n">
+        <v>46240</v>
+      </c>
+      <c r="K54" s="47" t="inlineStr">
+        <is>
+          <t>Per 3 Aug BOQ gap meeting decision (j). Going forward, SHD review meeting minutes will be traced via the Shop Drawing Tracker itself rather than a separate MOM doc — content for this specific MOM still pending from Shagun as of 6 Aug.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B55" s="46" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="C55" s="47" t="inlineStr">
+        <is>
+          <t>Develop a swatch sample-box presentation concept and show Khamille to decide how to move forward</t>
+        </is>
+      </c>
+      <c r="D55" s="47" t="inlineStr">
+        <is>
+          <t>Material Package FFE</t>
+        </is>
+      </c>
+      <c r="E55" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" s="47" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="G55" s="47" t="inlineStr">
+        <is>
+          <t>Khamille</t>
+        </is>
+      </c>
+      <c r="H55" s="47" t="n"/>
+      <c r="I55" s="46" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J55" s="53" t="n">
+        <v>46240</v>
+      </c>
+      <c r="K55" s="47" t="inlineStr">
+        <is>
+          <t>Per 4 Aug meeting with Khamille — swatch quantities/sizes agreed (already shared with H&amp;T, see Dev Log); spans both FFE and Fitout material packages. Decision on presentation approach expected by 7 Aug.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="46" t="n">
+        <v>46</v>
+      </c>
+      <c r="B56" s="46" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="C56" s="47" t="inlineStr">
+        <is>
+          <t>Compile all compliance documents received into a single consolidated record</t>
+        </is>
+      </c>
+      <c r="D56" s="47" t="inlineStr">
+        <is>
+          <t>Compliance Collection</t>
+        </is>
+      </c>
+      <c r="E56" s="46" t="n">
+        <v>2</v>
+      </c>
+      <c r="F56" s="47" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="G56" s="47" t="n"/>
+      <c r="H56" s="47" t="n"/>
+      <c r="I56" s="46" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J56" s="46" t="n"/>
+      <c r="K56" s="47" t="inlineStr">
+        <is>
+          <t>Per 3 Aug BOQ gap meeting. Ties to row above (Abdellatif compliance docs, target close 10 Aug).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A10:K47"/>
+  <autoFilter ref="A10:K56"/>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A4:B4"/>

</xml_diff>

<commit_message>
#newtask: install MCP for Woody to access Outlook (due 7 Aug)
</commit_message>
<xml_diff>
--- a/260730_K5M_Task Tracker.xlsx
+++ b/260730_K5M_Task Tracker.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Task Tracker'!$A$10:$K$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Task Tracker'!$A$10:$K$57</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -17,9 +17,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="16">
     <font>
       <name val="Calibri"/>
@@ -1046,7 +1044,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3215,8 +3213,53 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" s="46" t="n">
+        <v>47</v>
+      </c>
+      <c r="B57" s="46" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="C57" s="47" t="inlineStr">
+        <is>
+          <t>Install/authorize the MCP connector so Woody can read Shagun's Outlook inbox (read-only — no send capability)</t>
+        </is>
+      </c>
+      <c r="D57" s="47" t="inlineStr">
+        <is>
+          <t>WDCO Internal Project Management</t>
+        </is>
+      </c>
+      <c r="E57" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="F57" s="47" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="G57" s="47" t="n"/>
+      <c r="H57" s="47" t="n"/>
+      <c r="I57" s="46" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="J57" s="46" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="K57" s="47" t="inlineStr">
+        <is>
+          <t>Per #newtask. Type of Task guessed (Documentation) — doesn't cleanly fit the 7 categories, same issue as the SketchUp task. Depends on Shagun completing /mcp authorization herself. Feeds the new #GoodMorning/#checkmail mail-check design (see Command Center).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A10:K56"/>
+  <autoFilter ref="A10:K57"/>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A4:B4"/>

</xml_diff>

<commit_message>
Update MCP/Outlook task: tenant policy blocked, not just an auth step
</commit_message>
<xml_diff>
--- a/260730_K5M_Task Tracker.xlsx
+++ b/260730_K5M_Task Tracker.xlsx
@@ -3244,7 +3244,7 @@
       <c r="H57" s="47" t="n"/>
       <c r="I57" s="46" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>To Do</t>
         </is>
       </c>
       <c r="J57" s="46" t="inlineStr">
@@ -3254,7 +3254,7 @@
       </c>
       <c r="K57" s="47" t="inlineStr">
         <is>
-          <t>Per #newtask. Type of Task guessed (Documentation) — doesn't cleanly fit the 7 categories, same issue as the SketchUp task. Depends on Shagun completing /mcp authorization herself. Feeds the new #GoodMorning/#checkmail mail-check design (see Command Center).</t>
+          <t>Per #newtask. Type of Task guessed (Documentation) — doesn't cleanly fit the 7 categories, same issue as the SketchUp task. Depends on Shagun completing /mcp authorization herself. Feeds the new #GoodMorning/#checkmail mail-check design (see Command Center). Tested via the outlook-email-drafter connector (authenticated fine) — hit a hard tenant-level block: Access to OData is disabled, blocked by tenant Application Access Policy. This needs Wood Couture IT/M365 admin to exempt this app or grant mail-read consent at the admin level — not something fixable via personal authorization.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
#totalcheck: Woody upkeep — mark rows 14/38 Done, row 5 Stale (superseded), log validation-range gap
</commit_message>
<xml_diff>
--- a/260730_K5M_Task Tracker.xlsx
+++ b/260730_K5M_Task Tracker.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Tracker" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Task Tracker'!$A$10:$K$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Task Tracker'!$A$10:$K$58</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -1044,7 +1044,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1375,7 +1375,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1" thickBot="1">
+    <row r="15" hidden="1" ht="24" customHeight="1" thickBot="1">
       <c r="A15" s="49" t="n">
         <v>5</v>
       </c>
@@ -1406,13 +1406,13 @@
       <c r="H15" s="18" t="n"/>
       <c r="I15" s="9" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Stale</t>
         </is>
       </c>
       <c r="J15" s="9" t="n"/>
       <c r="K15" s="24" t="inlineStr">
         <is>
-          <t>Sent Ariel all details. Claire has asked to pause — new team joinee starts Monday (3 Aug); will assess if he can take this on before deciding who owns the work.</t>
+          <t>Sent Ariel all details. Claire has asked to pause — new team joinee starts Monday (3 Aug); will assess if he can take this on before deciding who owns the work. Superseded by S.No.31 ("Proceed with Ariel for required fit-out drawing updates; copy Resti") — same topic, decided at the 4 Aug meeting with Claire. Marked Stale + hidden by Woody, 6 Aug.</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1711,7 @@
       <c r="J22" s="10" t="inlineStr"/>
       <c r="K22" s="8" t="inlineStr">
         <is>
-          <t>Decided 3 Aug: full rebuild from scratch, once underlying data is fully verified/clean, rather than patching the 28 July v1. Freeze panes removed, Data tab rebuilt from canonical scope, and Hard Material partially updated as interim steps — but the ground-up rebuild is still the plan.</t>
+          <t>Decided 3 Aug: full rebuild from scratch, once underlying data is fully verified/clean, rather than patching the 28 July v1. Freeze panes removed, Data tab rebuilt from canonical scope, and Hard Material partially updated as interim steps — but the ground-up rebuild is still the plan. Update 6 Aug: the rebuild is visibly underway — Shagun's own new build, 260804_K5M_Internal Central COC.xlsx (Desktop, not yet in git), has 5 sheets (FFE_Main Data Sheet, Change Log, FFE_Fabrics, FFE_Hard Material, Shop Drawing Tracker) with real content populated, not just structure. Worth committing to git once she's ready.</t>
         </is>
       </c>
     </row>
@@ -1791,11 +1791,15 @@
       <c r="H24" s="18" t="n"/>
       <c r="I24" s="10" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J24" s="10" t="inlineStr"/>
-      <c r="K24" s="8" t="inlineStr"/>
+      <c r="K24" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Done — all 17 FFE items with a WDCO code now have SHD00 feedback collated (63 remarks total across Client/Internal/Factory review) in Shagun's new Central COC build (260804_K5M_Internal Central COC.xlsx, Desktop). All still marked unresolved (Value=False); 44 already have an Action/Action Owner noted.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="24" customHeight="1">
       <c r="A25" s="49" t="n">
@@ -2849,13 +2853,13 @@
       <c r="H48" s="47" t="n"/>
       <c r="I48" s="46" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="J48" s="46" t="n"/>
       <c r="K48" s="47" t="inlineStr">
         <is>
-          <t>Per 3 Aug BOQ gap meeting decision (a). Resti's raw calculation is complete (see row above) — this is writing it up clearly. References meetings/260803_K5M_Meeting_BOQ_Scope_Gap/post-meeting/Fit-out BOQ Scope Gap/stone_arch_findings.md.</t>
+          <t>Per 3 Aug BOQ gap meeting decision (a). Resti's raw calculation is complete (see row above) — this is writing it up clearly. References meetings/260803_K5M_Meeting_BOQ_Scope_Gap/post-meeting/Fit-out BOQ Scope Gap/stone_arch_findings.md. Done — reconciliation table rebuilt with Resti's numbers, confirmed by his clarifications (door-jamb depth doesn't affect the calc method; client's margin practice explains the 6&amp;7 gap, mirrored into 1&amp;2). All arches now resolved except the second banquette arch (confirmed not covered by any BOQ line).</t>
         </is>
       </c>
     </row>
@@ -3258,8 +3262,49 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" s="46" t="n">
+        <v>48</v>
+      </c>
+      <c r="B58" s="46" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="C58" s="47" t="inlineStr">
+        <is>
+          <t>Extend the Task Tracker's dropdown data validation (Umbrella Task/Priority/Type of Task/Status columns) beyond row 33 — every row added since (34 onward, including today's) has no validation at all</t>
+        </is>
+      </c>
+      <c r="D58" s="47" t="inlineStr">
+        <is>
+          <t>WDCO Internal Project Management</t>
+        </is>
+      </c>
+      <c r="E58" s="46" t="n">
+        <v>3</v>
+      </c>
+      <c r="F58" s="47" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="G58" s="47" t="n"/>
+      <c r="H58" s="47" t="n"/>
+      <c r="I58" s="46" t="inlineStr">
+        <is>
+          <t>To Do</t>
+        </is>
+      </c>
+      <c r="J58" s="46" t="n"/>
+      <c r="K58" s="47" t="inlineStr">
+        <is>
+          <t>Found during #totalcheck, 6 Aug, while fixing an invalid "Blocked" status value that the dropdown should have caught but didn't. Low priority — cosmetic/preventative, not blocking anything today.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A10:K57"/>
+  <autoFilter ref="A10:K58"/>
   <mergeCells count="3">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A4:B4"/>

</xml_diff>